<commit_message>
add 'detect_config_by_content' method to search keywords in sheets for mapping sheet names base on df values.
</commit_message>
<xml_diff>
--- a/extraction_script/data/1- ابلاغ بودجه مصوب سال 98.xlsx
+++ b/extraction_script/data/1- ابلاغ بودجه مصوب سال 98.xlsx
@@ -5,22 +5,35 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Armin KHoojavi\Downloads\persian-smart-accounting\extraction_script\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Armin KHoojavi\Downloads\persian-smart-accounting1\extraction_script\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A050E3C-9E09-4EDA-A1B1-9672A5EA87C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F563914-B9A2-44AE-B29E-BDDB68C39E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13035" yWindow="4455" windowWidth="15375" windowHeight="11505" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="16200" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ابلاغ_0" sheetId="1" r:id="rId1"/>
-    <sheet name="ابلاغ_1" sheetId="2" r:id="rId2"/>
-    <sheet name="ابلاغ_2" sheetId="3" r:id="rId3"/>
-    <sheet name="ابلاغ_3" sheetId="4" r:id="rId4"/>
-    <sheet name="ابلاغ_4" sheetId="5" r:id="rId5"/>
-    <sheet name="ابلاغ_5" sheetId="6" r:id="rId6"/>
+    <sheet name="0" sheetId="1" r:id="rId1"/>
+    <sheet name="1" sheetId="2" r:id="rId2"/>
+    <sheet name="2" sheetId="3" r:id="rId3"/>
+    <sheet name="3" sheetId="4" r:id="rId4"/>
+    <sheet name="4" sheetId="5" r:id="rId5"/>
+    <sheet name="5" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -322,12 +335,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -792,25 +805,25 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="7" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="7" t="s">
         <v>31</v>
       </c>
     </row>
@@ -970,7 +983,7 @@
       <c r="C9" s="2">
         <v>0</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="5" t="s">
         <v>32</v>
       </c>
       <c r="E9" s="6"/>
@@ -1354,7 +1367,7 @@
       <c r="D23" s="2">
         <v>145500</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="5" t="s">
         <v>32</v>
       </c>
       <c r="F23" s="6"/>
@@ -1552,7 +1565,7 @@
       <c r="A9" s="2">
         <v>6090</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="6"/>

</xml_diff>

<commit_message>
add 'detect_config_by_content' method to search keywords in sheets for mapping sheet names base on fuzzy search engine.
</commit_message>
<xml_diff>
--- a/extraction_script/data/1- ابلاغ بودجه مصوب سال 98.xlsx
+++ b/extraction_script/data/1- ابلاغ بودجه مصوب سال 98.xlsx
@@ -5,22 +5,35 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Armin KHoojavi\Downloads\persian-smart-accounting\extraction_script\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Armin KHoojavi\Downloads\persian-smart-accounting1\extraction_script\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A050E3C-9E09-4EDA-A1B1-9672A5EA87C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F563914-B9A2-44AE-B29E-BDDB68C39E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13035" yWindow="4455" windowWidth="15375" windowHeight="11505" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="16200" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ابلاغ_0" sheetId="1" r:id="rId1"/>
-    <sheet name="ابلاغ_1" sheetId="2" r:id="rId2"/>
-    <sheet name="ابلاغ_2" sheetId="3" r:id="rId3"/>
-    <sheet name="ابلاغ_3" sheetId="4" r:id="rId4"/>
-    <sheet name="ابلاغ_4" sheetId="5" r:id="rId5"/>
-    <sheet name="ابلاغ_5" sheetId="6" r:id="rId6"/>
+    <sheet name="0" sheetId="1" r:id="rId1"/>
+    <sheet name="1" sheetId="2" r:id="rId2"/>
+    <sheet name="2" sheetId="3" r:id="rId3"/>
+    <sheet name="3" sheetId="4" r:id="rId4"/>
+    <sheet name="4" sheetId="5" r:id="rId5"/>
+    <sheet name="5" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -322,12 +335,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -792,25 +805,25 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="7" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="7" t="s">
         <v>31</v>
       </c>
     </row>
@@ -970,7 +983,7 @@
       <c r="C9" s="2">
         <v>0</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="5" t="s">
         <v>32</v>
       </c>
       <c r="E9" s="6"/>
@@ -1354,7 +1367,7 @@
       <c r="D23" s="2">
         <v>145500</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="5" t="s">
         <v>32</v>
       </c>
       <c r="F23" s="6"/>
@@ -1552,7 +1565,7 @@
       <c r="A9" s="2">
         <v>6090</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="6"/>

</xml_diff>